<commit_message>
Font Awesome icons are working fine now.
</commit_message>
<xml_diff>
--- a/docs/Project tasks.xlsx
+++ b/docs/Project tasks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Webfejlesztes\portfolio\work4\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{248097A1-3F6C-4DEF-B76F-4E6BD5DC282B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A86525E2-B016-4AC8-811F-411C98AF03D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>Feladat szám</t>
   </si>
@@ -46,6 +46,15 @@
   </si>
   <si>
     <t>Különböző ágak létrehozása dev,test ágak.</t>
+  </si>
+  <si>
+    <t>Megfelelő betű típus beállítása.</t>
+  </si>
+  <si>
+    <t>Font-awesome beállítása az ikonok véget.</t>
+  </si>
+  <si>
+    <t>A dizájnon lévő összes kép letöltése.</t>
   </si>
 </sst>
 </file>
@@ -438,17 +447,26 @@
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7">
+      <c r="A7" s="2">
         <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
+      <c r="B8" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9">
+      <c r="A9" s="2">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
         <v>8</v>
       </c>
     </row>

</xml_diff>